<commit_message>
not sure why these aren't being ignored
</commit_message>
<xml_diff>
--- a/Incubations/Data/Conductivities.xlsx
+++ b/Incubations/Data/Conductivities.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carla López Lloreda\Dropbox\Grad school\Research\Humedales Puerto Rico\Incubations\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carla López Lloreda\Dropbox\Grad school\Research\Humedales Puerto Rico\PR-wetlands\incubations\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D1D333D-CE35-4B59-9AC5-3C6D12F8E300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C3313C-D5CC-4794-B91D-6968E82185EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{07CF8576-D001-473B-A347-F3778C328CFA}"/>
   </bookViews>
@@ -36,13 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>Sample</t>
-  </si>
-  <si>
-    <t>SpC (uS/cm)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="18">
   <si>
     <t>Sea water stock solution</t>
   </si>
@@ -71,16 +65,31 @@
     <t>Palmas 7/24/24</t>
   </si>
   <si>
-    <t>Cond</t>
-  </si>
-  <si>
-    <t>Temp (C)</t>
-  </si>
-  <si>
     <t>Palmas 8/17/24</t>
   </si>
   <si>
     <t>Tortuguero 8/16/24</t>
+  </si>
+  <si>
+    <t>period</t>
+  </si>
+  <si>
+    <t>summer</t>
+  </si>
+  <si>
+    <t>winter</t>
+  </si>
+  <si>
+    <t>spc_us_cm</t>
+  </si>
+  <si>
+    <t>cond</t>
+  </si>
+  <si>
+    <t>temp_C</t>
+  </si>
+  <si>
+    <t>sample</t>
   </si>
 </sst>
 </file>
@@ -452,113 +461,215 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17AA016C-FA9A-41D7-8C68-6D12EEAFD3E1}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C2">
+        <v>45208</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="C3">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="B2">
-        <v>45208</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="C4">
+        <v>2124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>978</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C5">
+        <v>3217</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="B4">
-        <v>2124</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C6">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="B5">
-        <v>3217</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="C7">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="B6">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C8">
+        <v>2791</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
         <v>7</v>
       </c>
-      <c r="B7">
-        <v>1644</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>2791</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="C10">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11">
+        <v>286.89999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" t="s">
         <v>10</v>
       </c>
-      <c r="B9">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>965</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="C12">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>13</v>
       </c>
-      <c r="B11">
-        <v>286.89999999999998</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12">
-        <v>955</v>
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13">
+        <v>443.6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>2318</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" t="s">
+        <v>5</v>
+      </c>
+      <c r="C17">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>2233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>